<commit_message>
Import terminale management missions into main workbook
Merge 45 terminale management missions from CSV into the main missions workbook and normalize XP values from difficulty so the import is immediately usable in admin.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/STMG_HUB_Missions_Programmes_Officiels.xlsx
+++ b/public/STMG_HUB_Missions_Programmes_Officiels.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2923,6 +2923,2751 @@
         <v>350</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MT1-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Ressources de Renault</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pour lancer sa nouvelle R5 E-Tech électrique, le groupe Renault a investi massivement dans son usine de Douai (Renault ElectriCity) et a déposé plusieurs brevets sur la motorisation. Les équipes de R&amp;D ont travaillé 3 ans sur le projet.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Identifiez et classez les ressources mobilisées par Renault pour ce projet de production.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ressources | tangibles | intangibles | production | innovation</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Ressources tangibles : financières (investissements massifs), matérielles (usine de Douai, chaînes de montage). Ressources intangibles : technologiques (brevets sur la motorisation), humaines (équipes R&amp;D, ingénieurs).</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MT1-02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Quels produits pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Démarche marketing Nespresso</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Nespresso a basé son succès sur la vente de dosettes de café premium via ses propres boutiques et son site web, répondant à une demande de café de haute qualité à domicile. Récemment, la marque a lancé la gamme Vertuo pour cibler les amateurs de cafés longs.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Caractérisez l'approche marketing de Nespresso lors du lancement de la gamme Vertuo.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>démarche marketing | besoins | offre | approche anticipatrice</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Nespresso adopte une approche marketing réactive et d'adaptation. L'entreprise a détecté une évolution des besoins des consommateurs (amateurs de cafés longs, notamment sur les marchés nord-américains et européens) et a ajusté son offre en créant une nouvelle technologie (Vertuo) pour y répondre et conserver ses parts de marché face à la concurrence.</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MT1-03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Comment assurer un fonctionnement cohérent ?</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Organisation du travail SNCF</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pour faire face aux pics de fréquentation lors des départs en vacances, la SNCF réorganise temporairement le travail de ses agents en gare (Gilets Rouges). Ces agents, habituellement assignés à des tâches administratives, sont déployés sur les quais pour orienter les voyageurs.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Repérez le mode d'organisation du travail mis en place par la SNCF pour répondre à cette contrainte.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>organisation du travail | flexibilité | polyvalence | ressources humaines</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>La SNCF met en place une organisation du travail basée sur la flexibilité fonctionnelle interne et la polyvalence. Les agents changent temporairement d'affectation pour répondre à une forte variation de l'activité, permettant à l'organisation d'être réactive sans avoir à recruter des contrats courts.</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MT1-04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Comment assurer un fonctionnement cohérent ?</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>4</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Coordination chez Decathlon</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Dans un grand magasin Decathlon, le directeur laisse une forte autonomie aux responsables de rayon (montagne, cycle, eau). Ces responsables se réunissent chaque lundi matin pour ajuster les opérations de la semaine et s'assurer que l'agencement global du magasin est cohérent.</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Analysez le principal mécanisme de coordination utilisé entre les responsables de rayon.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>coordination | ajustement mutuel | décentralisation | fonctionnement</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Le principal mécanisme de coordination est l'ajustement mutuel. Les responsables de rayon se coordonnent par le biais d'une communication informelle et de réunions régulières (le lundi) pour résoudre les problèmes d'agencement, ce qui est adapté à un mode de gestion décentralisé favorisant l'autonomie.</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MT1-05</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Quels choix d'organisation de la production ?</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Logistique Air France</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Air France gère quotidiennement des milliers de plateaux-repas pour ses vols. La compagnie a confié cette mission à Servair. Les repas doivent être livrés exactement 2 heures avant le décollage pour garantir la chaîne du froid et éviter les retards des avions.</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Identifiez le type de flux de production mis en place et montrez son enjeu pour l'organisation.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>logistique | flux tendus | chaîne logistique | qualité</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Il s'agit d'une production en flux tendus (ou juste-à-temps). L'enjeu est critique : la maîtrise de la chaîne logistique permet d'assurer la qualité du service (sécurité alimentaire) et d'éviter les coûts colossaux d'un retard de vol. Cela exige une coordination parfaite entre Air France et son sous-traitant.</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MT1-06</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Quels produits pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Modèle économique Danone</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Danone a réorienté son offre vers des produits végétaux (gamme Alpro) et la santé par l'alimentation. Les marges sur les produits végétaux sont nettement supérieures à celles des produits laitiers classiques, attirant une clientèle prête à payer plus cher pour des bénéfices santé.</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Analysez comment ce choix stratégique modifie le modèle économique et la création de valeur de Danone.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>modèle économique | création de valeur | positionnement | rentabilité</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Danone fait évoluer son business model en se positionnant sur un segment premium axé sur la santé (approche différenciatrice). La création de valeur financière est améliorée grâce à des marges unitaires plus fortes. La création de valeur perçue augmente car l'offre répond aux nouvelles attentes sociétales des consommateurs (bien-être, végétal).</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>MT1-07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, une chance pour la production ?</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>7</v>
+      </c>
+      <c r="G48" t="n">
+        <v>3</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Numérisation chez Michelin</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Michelin utilise l'intelligence artificielle pour analyser en temps réel les données de milliers de capteurs placés sur les machines de ses usines. L'algorithme anticipe les pannes avant qu'elles ne se produisent (maintenance prédictive).</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Diagnostiquez les avantages concurrentiels générés par l'utilisation de l'IA dans le processus de production de Michelin.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>transformation numérique | intelligence artificielle | processus | avantage concurrentiel</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>L'intégration de l'IA permet à Michelin de réaliser de la maintenance prédictive (innovation de procédé). Avantages : réduction drastique des arrêts de production non planifiés, optimisation des coûts de maintenance, allongement de la durée de vie des équipements et garantie d'une production continue pour répondre aux commandes, constituant un avantage concurrentiel par les coûts et la fiabilité.</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>MT1-08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>8</v>
+      </c>
+      <c r="G49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>GPEC chez Orange</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Avec le déploiement de la 5G et de la fibre, Orange anticipe la disparition progressive des anciens métiers liés au réseau cuivre (ADSL). Le groupe doit former des milliers de techniciens aux nouvelles technologies sous peine de manquer de main-d'œuvre qualifiée.</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Évaluez le rôle de la GPEC (Gestion Prévisionnelle des Emplois et des Compétences) pour accompagner cette transition technologique.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>GPEC | ressources humaines | compétences | anticipation | formation</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>La GPEC est vitale pour Orange afin d'adapter ses ressources humaines (intangibles) à sa stratégie technologique. Elle permet de diagnostiquer l'écart entre les compétences actuelles (réseau cuivre) et futures (5G/fibre). Son rôle est d'anticiper par un plan de formation interne massif (requalification) pour éviter des licenciements et garantir l'employabilité, tout en sécurisant la production de services.</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MT1-09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>9</v>
+      </c>
+      <c r="G50" t="n">
+        <v>3</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Financement L'Oréal</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Pour construire une nouvelle usine neutre en carbone en Europe, L'Oréal a besoin de 150 millions d'euros. Le groupe hésite entre utiliser ses importantes réserves de liquidités (autofinancement) ou recourir à un emprunt bancaire à des taux attractifs.</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Arbitrez entre ces deux modes de financement en justifiant votre choix au regard de la situation d'un grand groupe.</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>financement | investissement | autofinancement | emprunt | ressources financières</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>L'emprunt bancaire est souvent l'arbitrage privilégié si les taux d'intérêt sont bas (effet de levier positif), permettant à L'Oréal de conserver ses liquidités (autofinancement) pour d'autres opportunités stratégiques (rachat d'une startup, innovation). Cependant, l'autofinancement garantit une totale indépendance financière sans frais financiers. Une solution mixte (fonds propres + emprunt) est souvent la plus judicieuse pour répartir les risques.</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>MT1-10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Quels choix d'organisation de la production ?</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>10</v>
+      </c>
+      <c r="G51" t="n">
+        <v>4</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Externalisation Carrefour</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Carrefour constate que la gestion de sa gamme de plats préparés bio génère des coûts fixes très élevés dans ses propres usines, pesant sur la rentabilité. La direction envisage d'externaliser cette production à un sous-traitant spécialisé.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Proposez les critères de décision que Carrefour doit prendre en compte avant d'externaliser cette activité.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>organisation de la production | contrôle des coûts | externalisation | qualité</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Critères financiers : le coût complet de fabrication en interne vs le prix d'achat au sous-traitant. Critères qualitatifs : garantie du respect du cahier des charges bio et sécurité alimentaire. Critères stratégiques : le risque de perte de savoir-faire interne et la dépendance envers le fournisseur. Si le sous-traitant offre un coût spécifique plus bas avec une qualité certifiée, l'externalisation est pertinente.</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MT1-11</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Quels choix d'organisation de la production ?</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>11</v>
+      </c>
+      <c r="G52" t="n">
+        <v>4</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Flexibilité chez Zara</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Le succès de Zara (groupe Inditex) repose sur un modèle de production unique : renouveler les collections en boutique toutes les 3 semaines en s'appuyant sur des usines de proximité (Espagne, Portugal) capables de réagir instantanément aux ventes constatées.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Analysez la pertinence de cette gestion logistique (flux tendus) face aux caractéristiques du marché de la mode.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>logistique | flexibilité | réactivité | flux tendus</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Le marché de la mode est très volatil avec des cycles de vie de produits extrêmement courts. La production en flux poussés (produire de gros volumes à l'avance en Asie) engendre des invendus coûteux. Le choix de Zara (flux tendus et usines de proximité) garantit une hyper-réactivité, minimisant les coûts de stockage et les soldes. La pertinence est totale : la flexibilité devient le principal avantage concurrentiel.</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MT1-12</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Quels produits pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>12</v>
+      </c>
+      <c r="G53" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Business model BlaBlaCar</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>BlaBlaCar ne possède aucun véhicule ni chauffeur. Son rôle est de mettre en relation des conducteurs particuliers et des passagers via une plateforme numérique, en prélevant une commission sur chaque trajet réservé.</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Diagnostiquez le modèle économique de BlaBlaCar et montrez comment il génère de la création de valeur.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>modèle économique | plateforme | intermédiation | création de valeur</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Le modèle économique est un modèle de plateforme d'intermédiation (ou économie collaborative). La création de valeur financière provient des frais de service (commissions) sans supporter les coûts fixes de transport (pas de flotte à entretenir). La valeur perçue repose sur un service simple, sécurisé, économique pour les usagers et avec un fort impact environnemental positif (optimisation des sièges vides).</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>MT1-13</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>13</v>
+      </c>
+      <c r="G54" t="n">
+        <v>5</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Stratégie EDF</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>EDF doit démanteler ses anciennes centrales nucléaires et investir des milliards dans les énergies renouvelables (éolien, solaire) et les nouveaux réacteurs EPR, ce qui nécessite de modifier en profondeur son allocation de ressources sur les 20 prochaines années.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Construisez une argumentation justifiant les choix de restructuration des ressources tangibles et intangibles qu'EDF doit opérer pour réussir cette transition.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>décision stratégique | ressources | financement | investissement à long terme</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Argumentation : 1. Ressources financières : Les besoins d'investissement sont gigantesques. EDF devra mobiliser des financements externes (obligations vertes, soutien de l'État actionnaire). 2. Ressources intangibles : EDF doit pivoter d'une culture purement nucléaire vers les renouvelables (R&amp;D, rachat de brevets, GPEC pour former de nouveaux ingénieurs). 3. Ressources tangibles : Cession d'actifs vieillissants au profit de nouveaux parcs éoliens/solaires. La survie d'EDF dépend de sa capacité à piloter simultanément la fin de vie d'un outil industriel et l'émergence d'un nouveau, exigeant une réallocation totale du capital.</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MT1-14</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, une chance pour la production ?</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>14</v>
+      </c>
+      <c r="G55" t="n">
+        <v>5</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Workflow Doctolib</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Doctolib souhaite intégrer une nouvelle fonctionnalité : la pré-consultation numérique où un algorithme pose des questions médicales de base au patient avant son rendez-vous physique, afin de générer une fiche synthétique pour le médecin.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Formulez un diagnostic sur l'impact de ce nouveau flux de travaux (workflow) sur l'organisation du travail du médecin et la valeur perçue par le patient.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>workflow | transformation numérique | automatisation | santé</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Diagnostic : Pour le médecin (organisation du travail), ce workflow automatisé permet un gain de temps précieux lors de la consultation (suppression des questions administratives), favorisant un diagnostic plus rapide (efficience). Pour le patient (valeur perçue), cela donne un sentiment d'une prise en charge modernisée et personnalisée avant même le RDV. Cependant, le risque réside dans la déshumanisation du contact initial et la gestion sécurisée des données de santé très sensibles.</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MT1-15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Comment assurer un fonctionnement cohérent ?</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>15</v>
+      </c>
+      <c r="G56" t="n">
+        <v>5</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Réorganisation La Poste</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Face à la chute drastique du volume du courrier papier, La Poste transforme ses facteurs en livreurs de colis d'e-commerce et prestataires de services de proximité (visite aux personnes âgées, portage de repas).</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Élaborez les axes majeurs du plan d'action que la direction doit mener pour assurer le fonctionnement cohérent de cette nouvelle organisation du travail.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>organisation du travail | adaptation | polyvalence | stratégie de rupture</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Axes du plan d'action : 1. Ajustement des mécanismes de coordination : Les tournées doivent être repensées avec des outils numériques de routage en temps réel (standardisation des procédés par les algorithmes). 2. GPEC et formation : Accompagner les facteurs (enrichissement des tâches) pour développer des compétences relationnelles (services aux seniors) et logistiques (colis). 3. Adhésion : Communiquer sur le sens de cette mutation pour rassurer le personnel face au changement d'identité de leur métier historique, afin d'éviter une rupture du climat social.</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MT2-01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Culture d'entreprise Accor</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Le groupe hôtelier Accor promeut fortement le concept de 'Heartist' (contraction de Heart et Artist) auprès de ses collaborateurs. L'objectif est que chaque employé laisse s'exprimer sa personnalité pour offrir un accueil chaleureux et unique aux clients.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Identifiez la notion de management illustrée ici et précisez son utilité pour l'organisation.</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>culture de l'organisation | valeurs partagées | cohésion | implication</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Il s'agit de la culture de l'organisation. Promouvoir le concept de 'Heartist' permet de diffuser des valeurs partagées au sein des hôtels Accor. L'utilité est de fédérer les salariés autour d'une vision commune de l'hospitalité, d'augmenter leur implication au travail et de se différencier de la concurrence par une qualité de service unique.</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>MT2-02</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Intérêts des acteurs Mairie de Paris</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>La Mairie de Paris a décidé de piétonniser plusieurs grandes avenues. Les associations écologistes s'en félicitent, tandis que les commerçants locaux craignent une baisse de leur chiffre d'affaires due aux difficultés d'accès pour les clients motorisés.</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Caractérisez les relations entre ces différentes parties prenantes.</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>intérêts divergents | parties prenantes | acteurs externes | conflit</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Il s'agit d'une situation où les intérêts des acteurs externes sont divergents, voire conflictuels. L'association écologiste recherche une amélioration de la qualité de vie et de l'environnement (intérêt sociétal), alors que les commerçants poursuivent un objectif de rentabilité économique. La Mairie doit arbitrer et gérer ces tensions lors de sa prise de décision.</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>MT2-03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Style de direction Free / Iliad</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Xavier Niel, fondateur de Free, est connu pour prendre les décisions stratégiques finales de manière très directe. Il fixe le cap de manière audacieuse et exige de ses équipes des résultats rapides, tout en assumant seul la responsabilité des échecs.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Caractérisez le style de direction décrit dans cette situation.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>style de direction | leadership | autoritaire | prise de décision</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Le style de direction est principalement autoritaire (ou paternaliste / charismatique selon la proximité). Le pouvoir de décision est fortement centralisé autour de la personnalité du dirigeant fondateur. Ce style permet une grande réactivité et des décisions tranchées, bien adaptées à un marché des télécoms très agressif.</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>MT2-04</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>QVT chez Google France</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Google France offre à ses salariés des espaces de détente, des salles de sport gratuites, des repas sains à volonté et une grande flexibilité des horaires de travail. Les ingénieurs y passent de longues heures sans ressentir la pression traditionnelle.</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Analysez le lien entre ces dispositions de Qualité de Vie au Travail (QVT) et la performance recherchée par Google.</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>qualité de vie au travail | motivation | implication | performance sociale</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Google investit massivement dans la QVT pour répondre aux attentes de salariés très qualifiés. Ces avantages matériels et organisationnels sont des facteurs de motivation externes qui favorisent le bien-être. Un salarié épanoui est plus créatif, plus impliqué, et moins tenté de partir chez un concurrent (réduction du turnover). La performance sociale nourrit ici directement la performance de l'entreprise (innovation).</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MT2-05</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, vecteur d'amélioration de la relation clients ?</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Parcours client IKEA</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Un client d'IKEA peut configurer sa cuisine en 3D sur l'application mobile depuis chez lui, la sauvegarder sur son compte, puis venir en magasin pour qu'un vendeur affine le projet sur tablette avant de valider la commande.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Démontrez comment les outils numériques améliorent ici l'expérience d'achat du consommateur.</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>digitalisation | parcours client | interactivité | omnicanalité</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Le numérique permet la digitalisation du parcours client et crée une expérience omnicanale fluide (sans couture). Le client passe du virtuel (application) au physique (magasin) sans perdre ses données. Cela favorise l'interactivité, permet à l'entreprise de mieux connaître les besoins exacts du client, et au vendeur de conclure la vente avec un gain de temps considérable.</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MT2-06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, vecteur d'amélioration de la relation clients ?</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Administration électronique URSSAF</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>L'URSSAF a mis en place un portail 100% en ligne permettant aux auto-entrepreneurs de déclarer leur chiffre d'affaires et de payer leurs cotisations en trois clics chaque mois, remplaçant les formulaires papier.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Identifiez les avantages de cette administration électronique pour l'usager et pour l'organisme public.</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>administration électronique | simplification | usager | efficience</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Pour l'usager : simplification extrême des démarches, gain de temps, accessibilité 24h/24, traçabilité des paiements. Pour l'URSSAF : automatisation des processus, réduction massive des coûts de traitement papier, diminution des erreurs de saisie manuelle et recouvrement plus rapide des cotisations (efficience du service public).</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>MT2-07</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" t="n">
+        <v>3</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Communication interne Sanofi</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Lors de la fusion de deux départements de recherche, les équipes de Sanofi étaient démotivées par un sentiment d'opacité. La direction a lancé un réseau social d'entreprise interne et des webinaires hebdomadaires de questions-réponses avec le PDG.</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Diagnostiquez le rôle de cette stratégie de communication interne face à la situation de crise.</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>communication interne | adhésion | transparence | outils collaboratifs</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>La fusion a généré de l'anxiété et une perte de repères. La stratégie de communication interne (réseau social + webinaires) a un rôle fonctionnel de transparence et un rôle social d'adhésion. En permettant une communication descendante claire (les explications du PDG) et ascendante (les Q&amp;A des salariés), l'entreprise désamorce les rumeurs, restaure la confiance et favorise la cohésion des nouvelles équipes fusionnées.</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MT2-08</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>8</v>
+      </c>
+      <c r="G64" t="n">
+        <v>3</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Communication financière BNP Paribas</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>BNP Paribas publie chaque trimestre un rapport d'activité très détaillé, des infographies de synthèse sur son site web et organise des conférences téléphoniques avec les analystes financiers du monde entier.</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Identifiez les cibles de cette communication financière et expliquez l'importance stratégique de cette démarche.</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>communication financière | transparence | actionnaires | investisseurs</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Les cibles sont les acteurs financiers : actionnaires (actuels et potentiels), analystes boursiers, agences de notation et banques partenaires. L'enjeu est stratégique : une communication financière transparente, fiable et régulière permet de rassurer les marchés sur la santé de la banque, d'attirer des investisseurs, de soutenir le cours de l'action en bourse et de respecter les contraintes légales d'information financière.</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>MT2-09</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, vecteur d'amélioration de la relation clients ?</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>9</v>
+      </c>
+      <c r="G65" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Big Data Netflix</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>L'algorithme de Netflix analyse le temps de visionnage, les pauses, et les types de séries regardées par chaque utilisateur pour créer des recommandations hyper-personnalisées et même décider des futures séries à produire (comme House of Cards).</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Évaluez comment l'exploitation des traces numériques modifie la définition de l'offre chez Netflix.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>traces numériques | comportement du consommateur | big data | personnalisation</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Netflix passe d'une logique d'offre de masse à un marketing individualisé. L'exploitation intensive des traces numériques (Big Data) offre une connaissance client prédictive parfaite. Cela permet non seulement de personnaliser l'interface (fidélisation maximale), mais surtout de limiter le risque d'échec lors de la création de nouveaux produits, car l'offre est littéralement définie par les comportements constatés des abonnés.</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>MT2-10</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>10</v>
+      </c>
+      <c r="G66" t="n">
+        <v>4</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Travail collaboratif Airbus</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Airbus fabrique ses avions en répartissant la production entre l'Allemagne, l'Espagne, le Royaume-Uni et la France. Les ingénieurs doivent travailler simultanément sur les mêmes plans 3D sans jamais se rencontrer physiquement.</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Proposez et justifiez une solution d'outils de coopération pour surmonter cette contrainte géographique.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>coopération | outils collaboratifs | mode projet | intelligence collective</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Airbus doit déployer un environnement de travail collaboratif intégré (Cloud computing sécurisé et PLM - Product Lifecycle Management). Cela inclut des plateformes de partage de maquettes 3D en temps réel, des outils de messagerie instantanée, et des visioconférences immersives. Ces modes d'action coopératifs virtuels sont indispensables pour synchroniser les équipes (mode projet), partager l'intelligence collective et éviter les erreurs d'assemblage fatales entre pays.</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>MT2-11</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>11</v>
+      </c>
+      <c r="G67" t="n">
+        <v>4</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Fidélisation chez Ubisoft</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Les développeurs de jeux vidéo chez Ubisoft sont très sollicités par des studios concurrents américains offrant des salaires 30% plus élevés. Ubisoft ne peut pas s'aligner financièrement sur ces offres.</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Construisez un argumentaire managérial basé sur des facteurs de motivation alternatifs pour fidéliser ces talents.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>fidélisation | facteurs de motivation | qualité de vie au travail | rémunération</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Argumentaire : Si la rémunération (facteur externe) est plafonnée, Ubisoft doit miser sur les facteurs de motivation internes et la marque employeur. 1. Contenu du travail : offrir l'opportunité de travailler sur des franchises mondiales prestigieuses (Assassin's Creed) avec des technologies de pointe. 2. Ambiance et QVT : proposer une culture d'entreprise forte, créative, avec du télétravail flexible et des locaux innovants. 3. Évolution : garantir des formations continues et des parcours de carrière rapides vers des postes de Lead Designer.</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MT2-12</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>12</v>
+      </c>
+      <c r="G68" t="n">
+        <v>4</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Arbitrage TotalEnergies</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Lors d'une année de profits records, le conseil d'administration de TotalEnergies souhaite augmenter les dividendes versés aux actionnaires. Simultanément, les syndicats de salariés menacent de faire grève s'ils n'obtiennent pas d'augmentation générale des salaires face à l'inflation.</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Proposez une solution de gestion permettant à la direction de concilier ces attentes divergentes.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>intérêts divergents | conflit | actionnaires | salariés | arbitrage</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>La direction est face à un arbitrage classique entre performance financière (actionnaires) et performance sociale (salariés). Solution : Valider une hausse modérée des dividendes pour rassurer les marchés, et octroyer en parallèle une prime exceptionnelle de pouvoir d'achat (ou participation/intéressement) aux salariés. Lier l'effort financier aux résultats exceptionnels permet de récompenser les deux parties prenantes sans augmenter définitivement les coûts fixes (salaires de base).</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>MT2-13</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>13</v>
+      </c>
+      <c r="G69" t="n">
+        <v>5</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Gestion de crise Amazon</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Une enquête d'un grand média dénonce des conditions de travail dégradées et des destructions de produits neufs dans les entrepôts logistiques d'Amazon en France. La polémique s'enflamme sur les réseaux sociaux (bad buzz).</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Élaborez la stratégie de communication externe qu'Amazon doit déployer pour protéger sa e-réputation.</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>communication de crise | e-réputation | communication externe | bad buzz</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Stratégie de crise : 1. Réactivité : communiquer immédiatement (communiqué de presse) pour ne pas laisser le vide s'installer. 2. Transparence : reconnaître les faits avérés, contester les exagérations avec des chiffres précis. 3. Preuve (Earned/Owned media) : inviter la presse et des influenceurs à visiter des entrepôts pour montrer la réalité (journées portes ouvertes). 4. Actions correctives : annoncer publiquement de nouveaux partenariats avec des associations pour donner les invendus plutôt que de les détruire, transformant la crise en opportunité RSE.</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MT2-14</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, vecteur d'amélioration de la relation clients ?</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>14</v>
+      </c>
+      <c r="G70" t="n">
+        <v>5</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Stratégie omnicanale Sephora</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Sephora réalise d'excellents résultats sur son site e-commerce, mais observe une baisse de fréquentation physique de ses magasins. Le comité de direction hésite : fermer des magasins pour tout miser sur le web, ou réinvestir dans le réseau physique.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Argumentez en faveur du maintien et de la modernisation des boutiques physiques dans une logique d'expérience client globale.</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>omnicanalité | digitalisation de la relation client | expérience de consommation</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Argumentation : Fermer les boutiques serait une erreur car la cosmétique nécessite du test, du conseil humain et de l'expérience sensorielle. Sephora doit adopter une stratégie omnicanale où le physique et le digital se renforcent. Les boutiques doivent être digitalisées (miroirs virtuels, bornes de commande) et devenir des lieux d'expérience (masterclass maquillage, click &amp; collect). Le magasin physique n'est plus un simple lieu de stock, mais la vitrine événementielle de la marque employeur et de la relation client.</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MT2-15</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>15</v>
+      </c>
+      <c r="G71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Conduite du changement SNCF Réseau</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>SNCF Réseau doit faire face à l'ouverture à la concurrence européenne. Les agents historiques, attachés au monopole d'État, vivent cette transformation comme une menace pour leur statut et leur culture d'entreprise. Une grève dure se prépare.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Proposez un plan managérial systémique (direction, communication, QVT) pour fédérer les salariés autour de ce changement subi.</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>cohésion | conduite du changement | culture de l'organisation | dialogue social</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Plan systémique : 1. Direction et Dialogue social : Le management doit passer d'un style autoritaire/bureaucratique à un style consultatif. Organiser des tables rondes avec les syndicats pour co-construire les nouvelles méthodes de travail (éviter l'approche top-down). 2. Culture : Faire évoluer la culture interne en valorisant l'expertise historique des cheminots comme un atout concurrentiel face aux nouveaux entrants. 3. Communication interne et QVT : Rassurer sur le maintien des acquis fondamentaux, tout en finançant des formations massives pour monter en compétences. L'enjeu est de transformer la peur de la concurrence en défi collectif stimulant.</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MT3-01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Mécénat chez LVMH</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Le groupe LVMH a versé un don exceptionnel de 200 millions d'euros pour la reconstruction de la cathédrale Notre-Dame de Paris à la suite de l'incendie de 2019. Le groupe soutient également de nombreuses expositions artistiques.</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Identifiez cette pratique et déduisez-en l'objectif poursuivi par l'organisation envers la société.</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>mécénat | organisation civique | image | intérêt général</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Il s'agit d'une action de mécénat (soutien financier, humain ou matériel sans contrepartie directe explicite). LVMH s'inscrit ainsi comme une organisation civique. L'objectif est de participer à la préservation du patrimoine (intérêt général), tout en renforçant son image institutionnelle de leader français responsable, ancré dans l'art et l'histoire.</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>MT3-02</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Modes de consommation Vinted</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>L'application Vinted permet à des millions de particuliers de vendre et d'acheter des vêtements de seconde main directement depuis leur smartphone, contournant les magasins traditionnels d'habillement.</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Caractérisez ce nouveau mode de consommation qui bouleverse le secteur textile.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>modes de consommation | économie collaborative | économie circulaire</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Ce modèle repose sur l'économie collaborative (mise en relation de pair à pair via une plateforme) et l'économie circulaire (réemploi, seconde main, lutte contre le gaspillage). Ce changement de mode de vie, privilégiant l'usage et l'anti-consumérisme au neuf, s'impose aux marques de prêt-à-porter classiques qui voient leurs ventes baisser.</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>MT3-03</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, de nouvelles responsabilités ?</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>3</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Données personnelles CNIL</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Suite à une plainte, la CNIL a lourdement sanctionné une entreprise de e-commerce car cette dernière conservait les numéros de carte bancaire de ses clients sans leur consentement clair, dans une base de données mal sécurisée.</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Repérez le cadre réglementaire enfreint par l'entreprise et la nature de sa responsabilité.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>données personnelles | RGPD | protection | responsabilité</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>L'entreprise a enfreint le RGPD (Règlement Général sur la Protection des Données). L'organisation a manqué à sa responsabilité juridique et éthique de protection des données de ses usagers (défaut de consentement, défaut de sécurité), démontrant que la numérisation crée de strictes obligations de conformité.</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MT3-04</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>4</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Éthique Ben &amp; Jerry's</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>La marque de glaces Ben &amp; Jerry's s'approvisionne en cacao, sucre et vanille uniquement via le commerce équitable, garantissant un revenu décent aux petits producteurs mondiaux. Elle milite également activement pour les droits des réfugiés.</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Diagnostiquez la manière dont cette entreprise intègre l'éthique dans sa stratégie.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>éthique | RSE | commerce équitable | valeurs</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Ben &amp; Jerry's place l'éthique et la RSE au cœur de son business model. L'entreprise ne s'affranchit pas des questions de société, elle s'en empare (rémunération juste au Sud, militantisme). Ce n'est pas du simple 'social washing', car ces valeurs impactent directement sa chaîne d'approvisionnement (commerce équitable) et forgent une identité de marque militante fortement appréciée par sa cible.</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>MT3-05</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G76" t="n">
+        <v>2</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>L'application Yuka</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>L'application Yuka scanne les codes-barres des produits alimentaires pour évaluer leur impact sur la santé. Suite au succès de l'application, l'enseigne Intermarché a supprimé des dizaines d'additifs controversés de ses produits de marque distributeur.</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Expliquez comment le succès de cette application illustre l'évolution des rapports de force entre consommateurs et organisations.</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>modes de consommation | transparence | pouvoir du consommateur | adaptation</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Yuka illustre l'exigence croissante de transparence et de consommation responsable (alimentation saine). Le numérique donne un outil d'information puissant au consommateur, inversant le rapport de force. Les entreprises (comme Intermarché) sont contraintes de s'adapter très rapidement à ces nouveaux modes de vie pour éviter un boycott massif de leurs produits mal notés.</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>MT3-06</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>6</v>
+      </c>
+      <c r="G77" t="n">
+        <v>2</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Écosystème Aérospace Valley</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>À Toulouse, le pôle de compétitivité 'Aerospace Valley' regroupe le géant Airbus, des centaines de PME sous-traitantes, des écoles d'ingénieurs (ISAE-SUPAERO) et des laboratoires de recherche publics, tous géographiquement proches.</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Analysez l'intérêt pour une PME de s'implanter au sein de cette grappe d'entreprises (cluster).</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>écosystème | grappe d'entreprises | cluster | innovation | territoire</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>L'implantation dans ce cluster est un avantage stratégique. L'écosystème crée une synergie : la PME bénéficie d'un vivier de compétences (écoles), de partenariats de recherche, et d'un accès direct aux commandes d'Airbus. Cette proximité géographique et relationnelle stimule l'innovation collective et renforce la compétitivité de tout le territoire toulousain.</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MT3-07</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>7</v>
+      </c>
+      <c r="G78" t="n">
+        <v>3</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Égalité Société Générale</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>La Société Générale a mis en place un programme strict pour identifier et combler les écarts de salaires inexpliqués entre les hommes et les femmes à poste égal. De plus, elle impose qu'il y ait au moins 40% de femmes dans ses comités de direction.</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Diagnostiquez les enjeux de cette politique de lutte contre les discriminations pour la banque.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>discriminations | égalité hommes-femmes | éthique | RSE | attractivité</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>L'enjeu est triple. Juridique : se conformer à la loi (index égalité professionnelle). Éthique/Sociétal : répondre aux attentes de la société civile en matière de justice sociale, en corrigeant le 'plafond de verre' dans le secteur bancaire. RH/Managérial : la diversité dans les instances dirigeantes améliore la qualité de décision (diversité des profils) et renforce la marque employeur pour attirer des talents féminins de haut niveau.</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MT3-08</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, de nouvelles responsabilités ?</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>8</v>
+      </c>
+      <c r="G79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Algorithmes Criteo</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Criteo, fleuron technologique français, utilise des algorithmes complexes pour afficher des bannières publicitaires ciblées aux internautes en fonction de leur navigation passée. Des associations dénoncent l'opacité de ces outils de ciblage.</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Évaluez le risque éthique lié à l'utilisation de ces technologies et la responsabilité de l'entreprise.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>transparence des algorithmes | données personnelles | éthique | numérique</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Le ciblage comportemental soulève la question de la transparence des algorithmes (effet 'boîte noire'). Le risque éthique est la manipulation du consommateur à son insu et l'intrusion massive dans sa vie privée. La responsabilité de Criteo est d'expliquer de manière pédagogique le fonctionnement de ses algorithmes et de garantir le droit à l'opposition (opt-out), faute de quoi elle risque une perte de légitimité sociale.</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MT3-09</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>9</v>
+      </c>
+      <c r="G80" t="n">
+        <v>3</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Relocalisation Stellantis</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Le groupe automobile Stellantis (Peugeot-Fiat) a décidé de relocaliser la fabrication d'une partie de ses moteurs électriques en France, sur le site de Trémery (Moselle), après des années de délocalisation en Asie.</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Analysez les impacts croisés de cette décision stratégique d'implantation pour l'entreprise et pour le territoire local.</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>stratégie d'implantation | territoire | relocalisation | externalités positives</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Pour Stellantis : l'entreprise sécurise sa chaîne d'approvisionnement (moins de dépendance asiatique), raccourcit ses délais logistiques et bénéficie du label 'Fabriqué en France' très vendeur. Pour le territoire de Trémery : la relocalisation génère des externalités positives massives (maintien/création d'emplois industriels, rentrées fiscales pour la collectivité locale, dynamisation du tissu de sous-traitants régionaux). L'interaction est vertueuse.</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MT3-10</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>10</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Modèle Back Market</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Back Market est une plateforme française spécialisée dans la vente de smartphones et ordinateurs reconditionnés (réparés et remis à neuf). Elle connaît une croissance explosive face à l'achat de produits électroniques neufs.</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Argumentez en quoi le modèle d'affaires de Back Market est une réponse pertinente aux préoccupations écologiques de la société actuelle.</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>modes de consommation | économie circulaire | développement durable | obsolescence</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Argumentation : La société prend conscience de l'empreinte écologique désastreuse de l'électronique (extraction de métaux rares, e-déchets, obsolescence programmée). Back Market capte cette attente par l'économie circulaire : le produit est remis dans le circuit plutôt que jeté. L'entreprise crée de la valeur économique (forte croissance) tout en générant de la valeur écologique, offrant au consommateur responsable un acte d'achat déculpabilisant et moins cher.</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>MT3-11</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>11</v>
+      </c>
+      <c r="G82" t="n">
+        <v>4</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Pression sociétale McDonald's</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>McDonald's France fait face à de violentes critiques sur la quantité d'emballages jetables utilisés et sur la diététique de ses menus enfants. L'enseigne risque de perdre une grande partie de sa clientèle familiale soucieuse de l'environnement et de la santé.</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Proposez et justifiez un plan d'action RSE (Responsabilité Sociétale des Entreprises) pour McDonald's face à ces pressions.</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>RSE | pressions sociétales | éthique | image de marque</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Plan d'action RSE : 1. Environnement : Remplacer l'ensemble de la vaisselle jetable (plastique/carton) par de la vaisselle lavable et réutilisable pour la consommation sur place (action déjà amorcée par contrainte légale, mais à valoriser en communication). 2. Santé : Améliorer le 'Nutri-Score' des menus, baisser les taux de sel/sucre et proposer systématiquement des alternatives bio/végétales. L'enjeu vital est d'éviter le décrochage avec les normes sociétales (éviter d'être l'incarnation de la 'malbouffe polluante').</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>MT3-12</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Les transformations numériques, de nouvelles responsabilités ?</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>12</v>
+      </c>
+      <c r="G83" t="n">
+        <v>4</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Cybersécurité chez Ledger</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>L'entreprise française Ledger conçoit des portefeuilles physiques ultra-sécurisés (clés USB) pour protéger les cryptomonnaies de ses clients contre le piratage, dans un environnement numérique marqué par de fréquents piratages de plateformes d'échange.</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Évaluez comment la prise en compte des menaces du cyberespace constitue le cœur de la proposition de valeur de Ledger.</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>cybersécurité | blockchain | données stratégiques | protection</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Dans l'univers de la blockchain, le vol de données (clés privées) signifie la perte définitive de l'argent. La menace cyber est totale. Ledger ne vend pas qu'une clé USB, elle vend de la confiance et de la sécurité cryptographique absolue. Sa responsabilité de protection des données est son business model même. Son avantage concurrentiel mondial repose sur son expertise technologique garantissant l'inviolabilité du patrimoine numérique de ses clients.</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>MT3-13</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>13</v>
+      </c>
+      <c r="G84" t="n">
+        <v>5</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Arbitrage complexe Veolia</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Veolia exploite une usine d'incinération de déchets très rentable qui emploie 300 personnes dans un bassin peu dynamique. Cependant, les nouvelles normes environnementales révèlent que l'usine émet un niveau de pollution atmosphérique jugé nocif pour les riverains. La mise aux normes coûterait la moitié du chiffre d'affaires.</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Argumentez la décision stratégique que doit prendre le PDG en équilibrant les responsabilités économiques, sociales et environnementales de son groupe.</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>éthique | RSE | externalités négatives | arbitrage stratégique</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Argumentation : Veolia ne peut pas s'affranchir de ses externalités négatives (pollution). Ne rien faire engagerait sa responsabilité juridique et détruirait son image de champion de l'environnement (green washing). Fermer l'usine entraînerait un désastre social (300 chômeurs). Décision : Le PDG doit engager les travaux de mise aux normes, quitte à dégrader la rentabilité à court terme. Il doit négocier des aides avec l'État ou la région (écosystème) pour co-financer l'investissement, prouvant que la pérennité de l'entreprise repose sur un équilibre entre santé publique, emploi local et profitabilité.</t>
+        </is>
+      </c>
+      <c r="M84" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>MT3-14</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>14</v>
+      </c>
+      <c r="G85" t="n">
+        <v>5</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Partenariats Biocoop</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Le réseau de magasins bio Biocoop refuse d'acheter des produits cotés en bourse ou transportés par avion. L'enseigne souhaite développer de nouveaux magasins dans une région agricole, en exigeant que les gérants tissent des contrats équitables exclusifs avec des maraîchers locaux situés à moins de 150 km.</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Élaborez un diagnostic sur la manière dont Biocoop construit volontairement un écosystème d'affaires restrictif mais créateur de valeur.</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>écosystème d'affaires | partenariats | stratégie locale | valeurs</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Diagnostic : Biocoop rejette la logique de l'hypermarché globalisé. En imposant la proximité et l'équité, l'enseigne crée un écosystème d'affaires très intégré et territorialisé. C'est restrictif (moins de produits, pas de fruits hors saison) mais extrêmement puissant. Cela sécurise les revenus des producteurs partenaires (confiance, circuits courts) et crée une valeur d'estime inattaquable auprès d'une clientèle militante. L'entreprise structure son territoire et prouve que son modèle éthique est viable économiquement.</t>
+        </is>
+      </c>
+      <c r="M85" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>MT3-15</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>15</v>
+      </c>
+      <c r="G86" t="n">
+        <v>5</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Écosystème d'innovation Renault</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Pour produire ses futures voitures électriques, Renault a initié le pôle 'Software République' en s'associant avec des concurrents, des fournisseurs informatiques (Atos, Dassault Systèmes) et des instituts de recherche publics, partageant ainsi ses recherches sur la batterie et l'intelligence artificielle.</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Construisez un argumentaire démontrant que, face à la concurrence technologique (Tesla, constructeurs chinois), la survie d'une entreprise traditionnelle passe par la création d'un écosystème d'innovation ouvert plutôt que par le secret industriel.</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>écosystème d'innovation | coopération | compétitivité | alliances stratégiques</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Argumentaire : La voiture de demain est un 'ordinateur sur roues'. Renault, constructeur traditionnel, n'a pas les ressources financières ni le temps pour développer seul l'expertise logicielle, les puces et les batteries face aux géants américains et asiatiques (risques de rupture technologique). S'isoler dans le secret industriel serait fatal. La création d'un écosystème d'innovation (Software République) permet de mutualiser les risques financiers, de croiser des compétences ultra-spécialisées (synergie public/privé/tech) et d'accélérer la R&amp;D. La coopétition (coopérer avec des rivaux) devient la condition de survie de l'industrie européenne.</t>
+        </is>
+      </c>
+      <c r="M86" t="n">
+        <v>350</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 45 extra terminale management missions
Append the new management terminale mission set with unique IDs into the main workbook while keeping existing missions untouched, and keep the source CSV for traceability.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/STMG_HUB_Missions_Programmes_Officiels.xlsx
+++ b/public/STMG_HUB_Missions_Programmes_Officiels.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5668,6 +5668,2751 @@
         <v>350</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>MT1-16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>1.2. Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Définir le FRNG, BFR et la TN</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Le directeur financier de Sanofi analyse le bilan de l'entreprise pour préparer un nouvel investissement. Il a besoin de s'assurer de l'équilibre financier global de la structure avant d'emprunter.</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Définissez les notions de Fonds de Roulement Net Global (FRNG), Besoin en Fonds de Roulement (BFR) et Trésorerie Nette (TN).</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>FRNG | BFR | trésorerie nette | équilibre financier | définition</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Le FRNG représente l'excédent de ressources à long terme (capitaux propres, emprunts) après financement des actifs immobilisés. Le BFR est le besoin de financement généré par le cycle d'exploitation (stocks + créances - dettes fournisseurs). La TN est la différence entre le FRNG et le BFR : elle représente les liquidités réellement disponibles (si FRNG &gt; BFR).</t>
+        </is>
+      </c>
+      <c r="M87" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>MT1-17</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>1.3. Quels choix d'organisation de la production pour concilier flexibilité, qualité et maîtrise des coûts ?</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2</v>
+      </c>
+      <c r="G88" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Définir les méthodes de calcul de coûts</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>L'entreprise Renault fabrique plusieurs modèles de voitures dans son usine de Flins. La direction industrielle hésite sur la méthode comptable à utiliser pour évaluer la rentabilité d'un modèle spécifique.</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Définissez la méthode du coût complet et la méthode du coût spécifique.</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>coût complet | coût spécifique | charges directes | charges indirectes | définition</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Le coût complet consiste à imputer à un produit la totalité des charges (directes et indirectes) qu'il a générées, nécessitant des clés de répartition pour les charges communes. Le coût spécifique impute à un produit ses charges variables et uniquement les charges fixes directes qui lui sont propres, permettant de dégager une marge sur coût spécifique.</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>MT1-18</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>1.1. Quels produits ou quels services pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>3</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Indicateurs de création de valeur</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Le groupe LVMH présente son rapport annuel. Il y figure notamment le Chiffre d'Affaires, l'Excédent Brut d'Exploitation (EBE) et le Résultat Net.</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>À l'aide de ces indicateurs extraits du compte de résultat, expliquez comment l'entreprise mesure la création de valeur financière.</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>création de valeur | compte de résultat | indicateurs | valeur ajoutée | EBE</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>L'entreprise utilise les indicateurs du compte de résultat pour évaluer sa valeur financière. Le Chiffre d'Affaires mesure le volume des ventes. La Valeur Ajoutée (déduite des consommations intermédiaires) mesure la richesse réellement créée par son activité. L'EBE évalue la ressource tirée uniquement de l'exploitation, et le Résultat Net indique le bénéfice final (ou perte) distribuable ou mis en réserve.</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>MT1-19</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>1.2. Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>4</v>
+      </c>
+      <c r="G90" t="n">
+        <v>2</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Calcul simple de Trésorerie Nette</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>La maison Hermès dispose pour son dernier exercice d'un Fonds de Roulement Net Global (FRNG) de 500 millions d'euros et d'un Besoin en Fonds de Roulement (BFR) de 200 millions d'euros.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Calculez la Trésorerie Nette (TN) d'Hermès et interprétez ce résultat.</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>calcul | trésorerie nette | FRNG | BFR | analyse financière</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Calcul de la Trésorerie Nette : TN = FRNG - BFR. TN = 500 millions - 200 millions = 300 millions d'euros. Interprétation : La trésorerie nette est positive et très abondante. Hermès dégage un excédent de ressources à long terme largement suffisant pour couvrir ses besoins d'exploitation, ce qui témoigne d'une excellente santé financière et d'une forte capacité à investir ou à faire face aux imprévus.</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>MT1-20</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>1.3. Quels choix d'organisation de la production pour concilier flexibilité, qualité et maîtrise des coûts ?</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>5</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Pertinence du coût spécifique</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Air France étudie la rentabilité d'une ligne spécifique entre Paris et Tokyo. La compagnie identifie des charges variables (kérosène, repas) et des charges fixes directes (location de l'emplacement à l'aéroport de Tokyo).</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Analysez la pertinence de la méthode des coûts spécifiques pour décider du maintien ou non de cette ligne aérienne.</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>contrôle des coûts | coût spécifique | prise de décision | marge | charges fixes directes</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>La méthode des coûts spécifiques est très pertinente ici. Elle permet de calculer la marge sur coût spécifique en soustrayant du chiffre d'affaires de la ligne ses charges variables et ses charges fixes directes (location, personnel dédié). Si cette marge est positive, la ligne contribue à absorber les charges fixes communes d'Air France (siège social). Si elle est négative, la ligne détruit de la valeur et sa fermeture doit être envisagée.</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>MT1-21</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>1.3. Quels choix d'organisation de la production pour concilier flexibilité, qualité et maîtrise des coûts ?</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>6</v>
+      </c>
+      <c r="G92" t="n">
+        <v>2</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Logistique et flux tendus</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Decathlon approvisionne ses magasins européens à partir de ses entrepôts centraux. Pour certains produits très demandés (vélos), la production n'est lancée qu'une fois la commande magasin validée, afin de réduire les stocks.</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Identifiez ce mode d'organisation logistique et expliquez ses avantages pour l'entreprise.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>logistique | flux tendus | stockage | demande | réactivité</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Decathlon utilise ici la production en flux tendus (ou juste-à-temps), déclenchée par la demande (flux tirés). Les avantages sont une forte diminution des coûts liés au stockage (frais d'entrepôt, invendus, obsolescence) et une meilleure flexibilité, car la production s'adapte en temps réel aux besoins exacts des clients.</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>MT1-22</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>1.5. Comment assurer un fonctionnement cohérent des organisations ?</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>7</v>
+      </c>
+      <c r="G93" t="n">
+        <v>3</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Mécanismes de coordination</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Dans un centre d'appels Orange, les téléconseillers doivent suivre des scripts (scénarios) très précis pour chaque type d'appel client, et la durée maximale de chaque appel est paramétrée dans l'ordinateur.</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Identifiez le mécanisme de coordination mis en œuvre par Orange et précisez ses objectifs.</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>coordination | standardisation des procédés | procédures | contrôle</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Le mécanisme de coordination est la standardisation des procédés de travail (modèle de Mintzberg). Les étapes de l'action sont programmées à l'avance (scripts, durée imposée). L'objectif pour Orange est d'assurer une qualité de service uniforme, de faciliter la formation des nouveaux conseillers et de maximiser la productivité globale par le contrôle strict du temps.</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>MT1-23</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>1.4. Les transformations numériques, une chance pour la production ?</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>8</v>
+      </c>
+      <c r="G94" t="n">
+        <v>3</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Numérisation et objets connectés</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>L'usine Michelin de Clermont-Ferrand utilise des capteurs IoT (objets connectés) sur ses machines pour mesurer les vibrations et la température. Ces données remontent dans le Cloud pour être analysées en temps réel.</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Expliquez comment l'intégration de ces nouvelles technologies (objets connectés, cloud) améliore le processus de production.</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>transformations numériques | objets connectés | cloud computing | automatisation | maintenance</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Les objets connectés (IoT) permettent de collecter des données massives sur l'état des machines. L'informatique en nuage (Cloud) permet de stocker et d'analyser ces flux d'informations en temps réel. Cela améliore le processus de production en autorisant une maintenance prédictive : l'entreprise anticipe les pannes avant qu'elles ne surviennent, réduisant ainsi les arrêts coûteux des chaînes de fabrication.</t>
+        </is>
+      </c>
+      <c r="M94" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>MT1-24</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>1.1. Quels produits ou quels services pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>9</v>
+      </c>
+      <c r="G95" t="n">
+        <v>3</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Modèle économique Freemium</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Deezer propose une application d'écoute de musique. L'offre de base est gratuite mais comporte des publicités et des sauts de titres limités. L'offre Premium est payante et débloque toutes les fonctionnalités.</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Analysez ce modèle économique et montrez comment l'entreprise crée de la valeur avec l'offre gratuite.</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>modèle économique | freemium | création de valeur | publicité | conversion</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Deezer utilise un modèle économique 'Freemium' (contraction de free et premium). La création de valeur avec l'offre gratuite se fait indirectement : d'une part, grâce aux revenus générés par la vente d'espaces publicitaires, et d'autre part, en captant massivement des utilisateurs (effet de réseau) dont une partie finira par se convertir en abonnés payants pour améliorer leur expérience utilisateur.</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>MT1-25</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>1.2. Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>10</v>
+      </c>
+      <c r="G96" t="n">
+        <v>4</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Analyse du BFR négatif</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Carrefour encaisse quotidiennement l'argent de ses clients aux caisses (paiement comptant), alors que l'enseigne paie ses fournisseurs agroalimentaires à 60 jours. La rotation de ses stocks est très rapide.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Diagnostiquez l'impact de ce fonctionnement sur le Besoin en Fonds de Roulement (BFR) de Carrefour et sa Trésorerie Nette.</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>BFR négatif | ressources de financement | grande distribution | trésorerie nette</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>En encaissant ses clients avant de payer ses fournisseurs, et grâce à une rotation rapide des stocks, Carrefour génère des dettes d'exploitation supérieures à ses actifs d'exploitation. Le BFR est donc négatif : ce n'est plus un besoin de financement, mais une véritable 'ressource en fonds de roulement'. Cela impacte très positivement la Trésorerie Nette, qui devient abondante et permet à l'enseigne de placer cet argent ou d'autofinancer de nouveaux magasins sans emprunter.</t>
+        </is>
+      </c>
+      <c r="M96" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>MT1-26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>1.5. Comment assurer un fonctionnement cohérent des organisations ?</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>11</v>
+      </c>
+      <c r="G97" t="n">
+        <v>4</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Lean management et polyvalence</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Dans l'usine Toyota de Valenciennes, les ouvriers sont formés pour occuper plusieurs postes sur la chaîne de montage (polyvalence) et sont encouragés à arrêter la chaîne et proposer des solutions s'ils détectent un défaut.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Évaluez l'impact de cette organisation du travail (Lean management) sur la flexibilité et la qualité de la production.</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>organisation du travail | lean management | polyvalence | flexibilité | qualité</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Cette organisation (inspirée du Toyotisme et du Lean Management) s'oppose à la spécialisation extrême du Taylorisme. La polyvalence offre une grande flexibilité RH (remplacement immédiat en cas d'absence). Le fait de responsabiliser les ouvriers dans la détection des défauts (enrichissement des tâches) permet d'améliorer la qualité continue du produit final et de réduire les rebuts, tout en valorisant l'expertise du salarié.</t>
+        </is>
+      </c>
+      <c r="M97" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>MT1-27</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>1.1. Quels produits ou quels services pour quels besoins ?</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>12</v>
+      </c>
+      <c r="G98" t="n">
+        <v>4</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Innovation de procédé</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Air Liquide a modifié sa façon de produire de l'hydrogène industriel en intégrant une nouvelle technologie de capture du CO2 au sein même de ses usines, sans changer les caractéristiques du gaz vendu aux clients finaux.</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Qualifiez ce type d'innovation et justifiez l'intérêt pour l'organisation de mener ce type d'action stratégique.</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>innovation de procédé | méthode de production | impact environnemental | rentabilité</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Il s'agit d'une innovation de procédé. L'entreprise ne crée pas un nouveau produit, mais modifie considérablement la méthode de production. L'intérêt stratégique est double : réduire les coûts liés aux taxes carbone (maîtrise des coûts) et améliorer la performance environnementale du groupe (RSE), ce qui constitue un avantage concurrentiel face aux normes écologiques de plus en plus strictes.</t>
+        </is>
+      </c>
+      <c r="M98" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>MT1-28</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>1.2. Quelles ressources pour produire ?</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>13</v>
+      </c>
+      <c r="G99" t="n">
+        <v>5</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Arbitrage de financement</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Le groupe EDF doit financer la construction de six nouveaux réacteurs nucléaires EPR (coût estimé : plus de 50 milliards d'euros). Le groupe hésite entre l'autofinancement, un endettement massif ou une augmentation de capital avec l'aide de l'État.</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Construisez une argumentation pour aider la direction financière d'EDF à arbitrer entre ces trois ressources financières.</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>financement | investissement | ressources financières | augmentation de capital | endettement</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Argumentation : 1. L'autofinancement est impossible car les sommes (50 mds) dépassent largement les capacités des réserves d'EDF, et cela assécherait sa trésorerie. 2. L'emprunt bancaire classique (endettement massif) est très risqué car EDF est déjà lourdement endettée ; les charges d'intérêt dégraderaient fortement son résultat net. 3. L'augmentation de capital (fonds propres) soutenue par l'État est l'option la plus stratégique et soutenable. Elle renforce le FRNG sans créer de charges financières (pas d'intérêts), offrant la solidité nécessaire à un investissement sur très long terme (plus de 20 ans).</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>MT1-29</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>1.3. Quels choix d'organisation de la production pour concilier flexibilité, qualité et maîtrise des coûts ?</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>14</v>
+      </c>
+      <c r="G100" t="n">
+        <v>5</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Externalisation stratégique</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Airbus se concentre sur l'assemblage final des avions et la conception (R&amp;D). La fabrication de l'immense majorité des pièces (sièges, câblages, moteurs) est externalisée auprès de sous-traitants mondiaux spécialisés.</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Formulez un diagnostic critique de ce choix d'organisation de la production (Faire ou Faire faire).</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>externalisation | sous-traitance | contrôle des coûts | dépendance | stratégie</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Diagnostic : En choisissant le 'Faire faire' (externalisation), Airbus transforme des coûts fixes (usines) en coûts variables (achat de pièces). Cela accroît sa flexibilité financière et permet de bénéficier de l'expertise de pointe des sous-traitants. Cependant, cette stratégie présente des limites critiques : Airbus devient fortement dépendant de ses partenaires. Le moindre retard d'un sous-traitant (ou un défaut de qualité) peut paralyser toute la chaîne de montage finale, mettant en péril les délais de livraison et l'image du constructeur.</t>
+        </is>
+      </c>
+      <c r="M100" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>MT1-30</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Thème 1 : Les organisations et l'activité de production de biens et de services</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>1.5. Comment assurer un fonctionnement cohérent des organisations ?</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>15</v>
+      </c>
+      <c r="G101" t="n">
+        <v>5</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Diagnostic organisationnel complet</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>La Poste voit le volume de son courrier chuter. Pour s'adapter, elle développe la livraison de colis express et confie de nouveaux services aux facteurs (visite aux personnes âgées). Ces changements nécessitent de nouveaux outils numériques et des formations spécifiques.</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Élaborez un diagnostic systémique sur la manière dont La Poste doit faire évoluer la répartition des tâches, la coordination et la GPEC pour réussir ce virage stratégique.</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>organisation du travail | GPEC | coordination | adaptation | transformation</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Diagnostic systémique : 1. Répartition des tâches : Le métier de facteur s'enrichit (polyvalence). La Poste doit redéfinir les fiches de poste pour intégrer le commerce et le lien social. 2. Coordination : Les mécanismes passent d'une standardisation pure à un ajustement plus souple via des smartphones connectés gérant des tournées dynamiques. 3. GPEC (Ressources) : La Poste doit impérativement cartographier ses besoins futurs en compétences numériques et relationnelles, et déployer un plan de formation massif pour accompagner les agents historiques vers ces nouveaux métiers, garantissant ainsi l'adaptation aux besoins de l'organisation.</t>
+        </is>
+      </c>
+      <c r="M101" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>MT2-16</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" t="n">
+        <v>1</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Définir la culture d'organisation</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>L'entreprise alimentaire Michel et Augustin a créé une culture d'entreprise très forte : les employés sont appelés 'les trublions', les réunions se font dans des canapés, et le ton de l'entreprise se veut volontairement jeune, décalé et transparent.</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Définissez ce qu'est la culture d'une organisation et montrez son utilité dans ce contexte.</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>culture de l'organisation | valeurs partagées | rites | cohésion | identité</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>La culture d'une organisation est l'ensemble des valeurs, des normes, des mythes et des rituels (ici, le vocabulaire 'trublions', le ton décalé) partagés par l'ensemble de ses membres. Son utilité est fondamentale : elle fédère les acteurs autour d'une identité forte, favorise le sentiment d'appartenance (cohésion interne) et contribue à forger une 'marque employeur' attractive.</t>
+        </is>
+      </c>
+      <c r="M102" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>MT2-17</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Définir le style de direction</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Chez Tesla, le PDG Elon Musk impose directement ses visions techniques aux ingénieurs, fixe des délais souvent jugés irréalistes, et centralise la quasi-totalité des prises de décision stratégiques finales.</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Définissez ce qu'est un style de direction et qualifiez celui adopté dans cette situation.</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>style de direction | autoritaire | pouvoir de décision | centralisation</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Un style de direction définit la manière dont un dirigeant exerce le pouvoir, prend des décisions et interagit avec ses subordonnés. Ici, le style est autoritaire (ou directif). Le pouvoir de décision est extrêmement centralisé, la communication est descendante et la pression sur les résultats est forte, laissant peu d'autonomie formelle aux salariés.</t>
+        </is>
+      </c>
+      <c r="M103" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>MT2-18</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>3</v>
+      </c>
+      <c r="G104" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Définir l'e-réputation</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Sur les réseaux sociaux, Burger King France répond souvent aux critiques ou aux messages des internautes avec un humour sarcastique. L'entreprise surveille constamment ce qui se dit sur elle pour maîtriser son image en ligne.</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Définissez les notions d'identité numérique et d'e-réputation.</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>e-réputation | identité numérique | image | communication externe | réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>L'identité numérique correspond aux traces et aux contenus volontairement produits par l'organisation sur internet (sites, posts sur les réseaux sociaux). L'e-réputation, en revanche, est l'image perçue ou subie par l'organisation, construite à partir des avis, commentaires et rumeurs générés par les internautes. L'enjeu est d'aligner cette réputation subie avec l'identité voulue.</t>
+        </is>
+      </c>
+      <c r="M104" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>MT2-19</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>4</v>
+      </c>
+      <c r="G105" t="n">
+        <v>2</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Intérêts divergents SNCF</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>La direction de la SNCF annonce une réforme visant à modifier les critères d'avancement professionnel pour privilégier la performance individuelle. Les syndicats de cheminots, attachés à l'avancement à l'ancienneté, appellent à la grève.</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Caractérisez la nature des relations entre les acteurs dans cette organisation.</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>intérêts divergents | conflit social | acteurs internes | syndicats | direction</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Les relations sont conflictuelles en raison d'intérêts divergents entre les acteurs internes. La direction poursuit un objectif de performance et d'efficacité organisationnelle (logique de mérite). Les syndicats de salariés poursuivent un objectif de protection des acquis sociaux, de sécurité de l'emploi et d'équité collective (logique d'ancienneté). Cet antagonisme nécessite d'être régulé par le management et le dialogue social.</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>MT2-20</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2.2. Les transformations numériques, vecteur d'amélioration de la relation avec les clients et usagers ?</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>5</v>
+      </c>
+      <c r="G106" t="n">
+        <v>2</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Traces numériques Fnac</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Lorsqu'un client navigue sur le site de la Fnac en cherchant des appareils photo, le site mémorise son parcours. Lors de sa connexion suivante, le site lui affiche en page d'accueil des promotions ciblées sur des objectifs photographiques et des sacoches.</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Identifiez le procédé technique utilisé et expliquez en quoi il améliore la relation client.</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>traces numériques | digitalisation | personnalisation | données | parcours client</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>L'entreprise collecte et exploite les traces numériques (historique de navigation, cookies) laissées par le consommateur. Cela améliore la relation client en permettant une hyper-personnalisation de l'offre (Marketing One-to-One). Le client bénéficie de recommandations pertinentes qui facilitent son parcours d'achat, augmentant ainsi les chances de conversion et sa satisfaction.</t>
+        </is>
+      </c>
+      <c r="M106" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>MT2-21</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>6</v>
+      </c>
+      <c r="G107" t="n">
+        <v>2</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>QVT et motivation Doctolib</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Doctolib permet à 100% de ses salariés de faire du télétravail jusqu'à trois jours par semaine et finance une partie de l'équipement à domicile. La direction organise également des événements mensuels (team building).</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Analysez l'impact de ces mesures sur la motivation et la fidélisation des salariés.</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>qualité de vie au travail | motivation interne | télétravail | flexibilité | fidélisation</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Ces mesures agissent directement sur la Qualité de Vie au Travail (QVT) en offrant flexibilité et équilibre vie pro / vie perso. Le télétravail agit comme un puissant facteur de motivation (confiance, autonomie). L'organisation favorise ainsi l'implication de ses talents et limite le turn-over, la fidélisation étant un défi majeur dans le secteur très concurrentiel des technologies de la santé.</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>MT2-22</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>7</v>
+      </c>
+      <c r="G108" t="n">
+        <v>3</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Communication financière TotalEnergies</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>À la fin de chaque exercice, TotalEnergies publie un rapport annuel complet détaillant ses bénéfices, son plan d'affaires (business plan) à 5 ans pour la transition énergétique, et organise une réunion avec ses principaux actionnaires.</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Analysez l'importance stratégique de cette communication financière pour l'organisation.</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>communication financière | transparence | investisseurs | actionnaires | business plan</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>La communication financière est stratégique car elle s'adresse aux apporteurs de capitaux (actionnaires, banques, investisseurs). Le but n'est pas de vendre du pétrole, mais de vendre de la confiance. Le partage du business plan montre la solidité de la stratégie future. Une information transparente et normée permet de soutenir le cours en bourse et de faciliter les futurs financements de l'entreprise.</t>
+        </is>
+      </c>
+      <c r="M108" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>MT2-23</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>8</v>
+      </c>
+      <c r="G109" t="n">
+        <v>3</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Outils collaboratifs Dassault Systèmes</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Chez Dassault Systèmes, les développeurs utilisent un intranet et des espaces de travail virtuels collaboratifs pour concevoir de nouveaux logiciels de 3D. Ils partagent des codes, co-éditent des documents et interagissent via une messagerie instantanée interne sécurisée.</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Évaluez l'apport des outils numériques collaboratifs dans la mise en œuvre de la coopération au sein de l'organisation.</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>coopération | outils collaboratifs | intranet | modes d'action coopératifs | numérique</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>La coopération ne se décrète pas, elle nécessite des processus et des outils adaptés. L'apport des outils collaboratifs (intranet, messagerie) est de décloisonner l'entreprise, de permettre le travail asynchrone et à distance, et de faciliter le partage instantané des connaissances. Ils créent des interdépendances fluides entre les ingénieurs, constituant ainsi un levier indispensable pour l'innovation et l'efficacité des modes d'actions coopératifs.</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>MT2-24</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>9</v>
+      </c>
+      <c r="G110" t="n">
+        <v>3</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Marque employeur L'Oréal</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>L'Oréal a lancé une campagne de communication mondiale intitulée 'Freedom to go Beyond', avec des vidéos immersives sur YouTube et LinkedIn montrant le quotidien inspirant de ses jeunes chefs de produit et chercheurs.</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Identifiez le concept de communication RH illustré ici et expliquez ses objectifs vis-à-vis des acteurs externes.</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>marque employeur | recrutement | communication RH | image | attractivité</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Il s'agit du concept de 'Marque employeur' (employer branding). L'objectif de L'Oréal n'est pas de communiquer sur ses cosmétiques (com' commerciale), mais de valoriser son image en tant que lieu de travail attractif. Vis-à-vis des acteurs externes (les jeunes diplômés et futurs talents), cette communication vise à séduire, à se différencier des concurrents et à faciliter les futures campagnes de recrutement de profils de haut niveau.</t>
+        </is>
+      </c>
+      <c r="M110" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>MT2-25</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2.2. Les transformations numériques, vecteur d'amélioration de la relation avec les clients et usagers ?</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>10</v>
+      </c>
+      <c r="G111" t="n">
+        <v>4</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Digitalisation parcours client Sephora</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Sephora a équipé ses vendeurs en magasin de terminaux tactiles permettant de retrouver l'historique d'achat en ligne du client. Le client peut aussi utiliser un miroir virtuel en réalité augmentée pour essayer virtuellement du maquillage.</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Diagnostiquez les avantages de cette digitalisation du parcours client pour le consommateur et pour l'organisation.</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>digitalisation | expérience client | omnicanalité | innovation | personnalisation</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Pour le consommateur : la valeur perçue augmente considérablement grâce à une expérience ludique (miroir) et un service sans couture (le vendeur connaît ses goûts). C'est une omnicanalité parfaite. Pour Sephora : l'organisation collecte de nouvelles données comportementales, modernise son image de marque, fluidifie le passage en caisse et augmente très fortement ses taux de conversion en magasin (chiffre d'affaires).</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>MT2-26</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>11</v>
+      </c>
+      <c r="G112" t="n">
+        <v>4</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Stratégie de communication globale Decathlon</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Pour lancer une nouvelle tente de camping, Decathlon achète des spots publicitaires à la TV (Paid Media), publie des tutoriels de montage sur son propre site web (Owned Media) et espère que les campeurs partageront leurs vidéos d'utilisation sur TikTok (Earned Media).</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Analysez la pertinence de cette approche POEM (Paid, Owned, Earned Media) pour la stratégie de communication globale de Decathlon.</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>communication globale | POEM | publicité | réseaux sociaux | e-réputation</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>L'approche POEM est très pertinente car elle crée une communication globale et intégrée. Le 'Paid Media' (TV) assure une forte visibilité de masse immédiate. Le 'Owned Media' (site web) garantit une information maîtrisée et experte (réassurance du client). Le 'Earned Media' (TikTok) apporte la caution des pairs et la viralité, renforçant la crédibilité du produit par le bouche-à-oreille numérique, le tout optimisant le budget communication de la marque.</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>MT2-27</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>12</v>
+      </c>
+      <c r="G113" t="n">
+        <v>4</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Facteurs de motivation Ubisoft</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Chez Ubisoft, éditeur de jeux vidéo, les augmentations de salaires sont limitées. Pour compenser, la direction offre à ses développeurs des jours de temps libre pour travailler sur des projets personnels créatifs, et organise des concours internes de création.</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Démontrez pourquoi l'entreprise privilégie les facteurs de motivation internes face aux limites de la rémunération (facteur externe).</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>motivation | facteurs internes | facteurs externes | reconnaissance | implication</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>La rémunération (facteur externe) est un levier limité financièrement et dont l'effet motivant s'estompe vite. Ubisoft privilégie les facteurs internes de motivation liés au contenu même du travail : l'autonomie, l'enrichissement des tâches et la stimulation intellectuelle (concours, projets perso). Ces facteurs répondent au besoin d'accomplissement de ces profils créatifs, générant une implication profonde et une fidélisation que l'argent seul ne peut garantir.</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>MT2-28</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>13</v>
+      </c>
+      <c r="G114" t="n">
+        <v>5</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Gestion de crise Lactalis</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>L'entreprise Lactalis fait face à un scandale sanitaire (lait infantile contaminé). Au début de la crise, l'entreprise communique très peu et refuse de répondre aux journalistes, ce qui déclenche un 'bad buzz' retentissant sur les réseaux sociaux et un effondrement de la confiance client.</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Élaborez un diagnostic critique de cette gestion de crise et proposez les axes d'une communication externe corrective appropriée.</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>communication de crise | bad buzz | e-réputation | transparence | confiance</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Diagnostic : La stratégie du silence de Lactalis est un échec majeur en gestion de crise. L'absence de communication officielle laisse le champ libre aux rumeurs et aux réseaux sociaux (bad buzz), détruisant l'e-réputation et l'image de marque. Axes correctifs : 1. Communication immédiate et transparente : le PDG doit s'exprimer publiquement, assumer la responsabilité et présenter des excuses. 2. Preuve d'action : annoncer le rappel immédiat des produits et l'ouverture d'une enquête indépendante. L'enjeu est de restaurer la confiance perdue des consommateurs.</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>MT2-29</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2.1. Comment fédérer les acteurs de l'organisation ?</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>14</v>
+      </c>
+      <c r="G115" t="n">
+        <v>5</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Arbitrage complexe Stellantis</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Après une année record, Stellantis distribue d'importants dividendes à ses actionnaires. Simultanément, la direction refuse une augmentation des salaires de base aux ouvriers, invoquant la nécessité d'investir dans l'électrique. Les syndicats bloquent plusieurs usines stratégiques.</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Construisez une argumentation managériale pour aider la direction à arbitrer ce conflit et à réaligner les intérêts divergents sans compromettre la stratégie à long terme.</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>conflit social | intérêts divergents | arbitrage | dialogue social | actionnaires</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Argumentation : La direction fait face à un blocage qui menace la production immédiate. Arbitrer uniquement en faveur des actionnaires (dividendes) détruit le climat social. Arbitrer uniquement par une forte hausse des salaires fixes grève les capacités d'investissement (électrique). La solution passe par le dialogue social et le compromis : la direction doit lier la rémunération à la performance exceptionnelle via des dispositifs collectifs (primes d'intéressement, participation). Cela permet de récompenser l'effort des salariés à l'instant T tout en préservant la structure des coûts fixes à long terme.</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>MT2-30</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Thème 2 : Les organisations et les acteurs</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2.3. Communique-t-on de la même manière avec tous les acteurs ?</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>15</v>
+      </c>
+      <c r="G116" t="n">
+        <v>5</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Plan de communication global Accor</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Le groupe hôtelier Accor lance une initiative majeure : supprimer tous les plastiques à usage unique de ses hôtels dans le monde. Ce projet implique les fournisseurs, les 260 000 collaborateurs et les clients finaux.</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Concevez la stratégie de communication globale et intégrée (ascendante, descendante et externe) nécessaire pour assurer le succès de cette initiative.</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>communication globale | communication interne | communication externe | RSE | adhésion</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Stratégie globale : 1. Communication interne descendante : Une note du PDG via l'intranet expliquant les objectifs RSE de l'entreprise pour donner le cap. 2. Communication interne ascendante/horizontale : Mettre en place des boîtes à idées ou forums sur le RSE (Réseau Social d'Entreprise) pour que le personnel de terrain propose des solutions de remplacement du plastique (adhésion). 3. Communication externe : Campagne sur les réseaux sociaux et affichages dans les chambres pour informer les clients de cette politique écoresponsable, valorisant ainsi l'image de marque du groupe auprès de son écosystème.</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>MT3-16</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>1</v>
+      </c>
+      <c r="G117" t="n">
+        <v>1</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Définir la Déontologie et l'Éthique</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Les employés de la banque Société Générale doivent signer un code de bonne conduite qui leur interdit formellement d'utiliser les informations financières de leurs clients à des fins d'enrichissement personnel.</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Définissez les notions d'éthique et de déontologie dans le contexte des affaires.</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>éthique | déontologie | règles de conduite | transparence | responsabilité</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>L'éthique est une réflexion morale sur les valeurs et les principes (bien/mal, juste/injuste) qui guident l'action d'une entreprise dans la société. La déontologie est l'ensemble des règles, des devoirs et des obligations professionnelles, souvent formalisés dans une charte ou un code de conduite, que doivent respecter les collaborateurs d'une organisation dans l'exercice de leur métier.</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>MT3-17</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>2</v>
+      </c>
+      <c r="G118" t="n">
+        <v>1</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Définir le Greenwashing</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>La marque H&amp;M a lancé une collection 'Conscious' avec des étiquettes vertes, tout en continuant à produire des millions de vêtements à bas coût dans des pays en voie de développement (fast-fashion). Des ONG accusent la marque de tromperie.</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Définissez le concept de 'greenwashing' (écoblanchiment).</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>greenwashing | RSE | communication | éthique | image trompeuse</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Le greenwashing (ou écoblanchiment) est une pratique de communication trompeuse utilisée par une organisation. Elle consiste à verdir artificiellement son image et à mettre en avant des arguments écologiques ou de développement durable, alors que la réalité de ses pratiques de production et de son modèle économique reste polluante ou non éthique.</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>MT3-18</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>3</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Définir le mécénat</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>La Fondation TotalEnergies finance chaque année des programmes de restauration de monuments historiques en France et des bourses pour l'éducation des jeunes issus de milieux défavorisés.</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Définissez le mécénat et précisez son but principal par rapport au sponsoring (parrainage).</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>mécénat | fondation | intérêt général | organisation civique | image institutionnelle</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Le mécénat est le soutien matériel, humain ou financier apporté sans contrepartie publicitaire directe à une œuvre ou une personne pour l'exercice d'activités d'intérêt général (culture, éducation, solidarité). À la différence du sponsoring qui vise des retombées commerciales directes, le mécénat relève du rôle civique de l'organisation et vise à asseoir son image institutionnelle sur le long terme.</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>MT3-19</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>4</v>
+      </c>
+      <c r="G120" t="n">
+        <v>2</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Discriminations et Égalité Kering</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Le groupe de luxe Kering (Gucci, YSL) publie chaque année son index de l'égalité professionnelle et a mis en place un congé paternité de 14 semaines payé à 100 % dans le monde entier pour réduire les biais de recrutement liés à la maternité.</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Analysez l'enjeu de cette lutte contre les discriminations dans les relations de travail.</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>discriminations | égalité hommes-femmes | RSE | éthique | marque employeur</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>L'enjeu est à la fois éthique, légal et managérial. Éthiquement, l'organisation s'engage concrètement pour l'égalité femmes-hommes. Sur le plan managérial, supprimer le 'risque maternité' lors des recrutements garantit que Kering attire et promeut les meilleurs talents uniquement sur leurs compétences. Cela renforce puissamment la marque employeur et la cohésion interne.</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>MT3-20</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>3.2. Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>5</v>
+      </c>
+      <c r="G121" t="n">
+        <v>2</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Économie de la fonctionnalité Michelin</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Michelin propose à de grandes flottes de camions de ne plus acheter leurs pneus, mais de payer un abonnement calculé selon le nombre de kilomètres parcourus. Michelin reste propriétaire des pneus et se charge de l'entretien.</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Identifiez ce nouveau modèle économique et montrez en quoi il répond aux évolutions de la société.</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>économie de la fonctionnalité | usage | services | développement durable | modes de consommation</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Il s'agit de l'économie de la fonctionnalité, qui privilégie la vente de l'usage d'un bien plutôt que sa propriété. Ce changement de mode de consommation répond aux enjeux de développement durable : Michelin a tout intérêt à fabriquer des pneus très résistants et à les rechapables pour maximiser ses marges, luttant ainsi mécaniquement contre le gaspillage et l'obsolescence programmée.</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>MT3-21</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>3.3. Les transformations numériques, de nouvelles responsabilités pour les organisations ?</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>6</v>
+      </c>
+      <c r="G122" t="n">
+        <v>2</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>RGPD et données Cdiscount</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Le site de e-commerce Cdiscount collecte des millions de données (nom, adresse, historique d'achats). Suite à l'application du RGPD européen, l'entreprise a dû nommer un DPO (Délégué à la Protection des Données) et instaurer des pop-ups de consentement clairs.</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Précisez l'obligation légale illustrée ici et les risques encourus par l'organisation en cas de non-respect.</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>données personnelles | RGPD | sécurité | confidentialité | sanctions</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>L'organisation a l'obligation légale de protéger les données personnelles de ses clients, d'en garantir la confidentialité et d'obtenir leur consentement explicite (règles du RGPD). En cas de manquement ou de fuite de données, l'entreprise s'expose à de très lourdes sanctions financières de la CNIL (jusqu'à 4% du CA mondial) et à une destruction irrémédiable de son image de marque.</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>MT3-22</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>3.4. Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>7</v>
+      </c>
+      <c r="G123" t="n">
+        <v>3</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Pôle de compétitivité Aerospace Valley</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>À Toulouse, le cluster 'Aerospace Valley' regroupe Airbus, de nombreuses PME sous-traitantes de l'aéronautique, l'école d'ingénieurs ISAE-SUPAERO, et reçoit des financements de la Région Occitanie.</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Diagnostiquez les avantages de cette proximité géographique (écosystème territorial) pour les organisations impliquées.</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>écosystème d'innovation | grappe d'entreprises | cluster | territoire | compétitivité</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Cette concentration d'acteurs (cluster ou grappe d'entreprises) crée de fortes externalités positives. Airbus trouve un vivier de sous-traitants réactifs et qualifiés. Les PME accèdent à des donneurs d'ordres mondiaux. Les écoles forment des ingénieurs directement employables. Cette synergie d'écosystème favorise le partage des savoirs, l'innovation collective et renforce l'attractivité et la compétitivité économique de tout le territoire toulousain.</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>MT3-23</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>3.3. Les transformations numériques, de nouvelles responsabilités pour les organisations ?</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>8</v>
+      </c>
+      <c r="G124" t="n">
+        <v>3</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Blockchain et traçabilité Carrefour</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Carrefour utilise la technologie de la blockchain (chaîne de blocs) pour tracer l'intégralité du parcours d'un poulet fermier. En scannant un QR code en magasin, le consommateur accède à des données infalsifiables sur le lieu d'élevage, l'alimentation et la date d'abattage.</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Expliquez comment cette technologie numérique permet à l'entreprise de répondre à une préoccupation de la société.</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>blockchain | traçabilité | transparence | sécurité alimentaire | numérique</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>La société exige de plus en plus de transparence et de sécurité alimentaire (modes de consommation). La blockchain est une technologie de stockage et de transmission d'informations transparente, sécurisée et décentralisée. Son caractère infalsifiable permet à Carrefour d'offrir une garantie de traçabilité absolue, rassurant le consommateur et se démarquant éthiquement de ses concurrents par la preuve technologique.</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>MT3-24</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>3.2. Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>9</v>
+      </c>
+      <c r="G125" t="n">
+        <v>3</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Économie circulaire Back Market</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Back Market ne vend aucun produit électronique neuf. La plateforme française met en relation des reconditionneurs professionnels et des consommateurs pour donner une seconde vie aux smartphones et ordinateurs.</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Démontrez en quoi le modèle de cette entreprise s'inscrit dans les attentes écologiques de la société actuelle.</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>économie circulaire | modes de consommation | développement durable | obsolescence | plateforme</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Face aux préoccupations climatiques et à la dénonciation de l'obsolescence programmée des appareils électroniques (gaspillage, métaux rares), Back Market a bâti son modèle sur l'économie circulaire. Plutôt que la destruction (modèle linéaire), l'entreprise favorise la réparation et le réemploi. Elle capte ainsi l'attente d'une consommation plus responsable et durable, tout en offrant un avantage prix au client.</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>MT3-25</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>3.4. Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>10</v>
+      </c>
+      <c r="G126" t="n">
+        <v>4</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Stratégie d'implantation Le Slip Français</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>L'entreprise textile Le Slip Français a fait le choix stratégique de fabriquer 100% de ses produits en France, en s'appuyant sur un réseau de PME partenaires réparties dans différentes régions françaises, alors que ses concurrents produisent en Asie.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Évaluez les effets de cette stratégie d'implantation sur l'écosystème local et sur l'image de l'organisation.</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>stratégie d'implantation | relocalisation | écosystème | tissu économique | image de marque</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Effets sur l'écosystème local : l'organisation dynamise le territoire en maintenant ou créant des emplois industriels, et soutient la survie d'un savoir-faire textile français menacé. Effets sur l'image : cette démarche de relocalisation est l'ADN de la marque. Bien que ses coûts de production soient plus élevés, elle crée une immense valeur perçue éthique et civique, justifiant un prix de vente premium auprès de consommateurs militants.</t>
+        </is>
+      </c>
+      <c r="M126" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MT3-26</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>3.3. Les transformations numériques, de nouvelles responsabilités pour les organisations ?</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>11</v>
+      </c>
+      <c r="G127" t="n">
+        <v>4</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Transparence des algorithmes Parcoursup</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Le Ministère de l'Enseignement Supérieur a été contraint, sous la pression d'associations et d'étudiants, de rendre publics les codes sources des algorithmes locaux utilisés par certaines universités pour trier les dossiers des candidats sur la plateforme Parcoursup.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Analysez l'enjeu sociétal majeur que soulève le traitement des données par ce type d'algorithme public.</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>transparence des algorithmes | administration publique | équité | biais | données</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>L'automatisation des processus de décision (orientation de milliers de jeunes) par des algorithmes pose un enjeu démocratique d'équité. L'opacité (l'effet 'boîte noire') génère de la défiance et des suspicions de biais sociaux ou géographiques. La transparence des algorithmes est une nouvelle responsabilité incontournable pour l'administration publique : elle seule permet de garantir que les critères de sélection soient audités, justes et non discriminatoires.</t>
+        </is>
+      </c>
+      <c r="M127" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>MT3-27</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>3.2. Les changements de modes de vie s'imposent-ils aux organisations ?</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>12</v>
+      </c>
+      <c r="G128" t="n">
+        <v>4</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Économie collaborative BlaBlaCar</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Face au coût élevé des trajets en train et à l'usage individuel de la voiture, BlaBlaCar a popularisé le covoiturage en France. Aujourd'hui, l'entreprise diversifie son offre avec BlaBlaCar Daily pour les trajets quotidiens domicile-travail.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Expliquez comment cette organisation a su transformer une évolution des rapports sociaux en un modèle économique pérenne.</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>économie collaborative | plateforme | covoiturage | modes de vie | mobilité</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>BlaBlaCar a capté le passage d'une société de la possession (avoir sa voiture) à une société du partage et de la fonctionnalité (économie collaborative). En numérisant la mise en relation (la plateforme), l'entreprise a monétisé le partage des frais de transport. En s'attaquant désormais aux trajets quotidiens, elle s'adapte à un nouveau besoin sociétal massif (congestion urbaine, pouvoir d'achat, écologie) en devenant un acteur global de la mobilité partagée.</t>
+        </is>
+      </c>
+      <c r="M128" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>MT3-28</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>13</v>
+      </c>
+      <c r="G129" t="n">
+        <v>5</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Entreprise à mission Danone</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Sous l'impulsion de son ancien PDG Emmanuel Faber, Danone est devenue la première grande entreprise française cotée en Bourse à adopter le statut d''Entreprise à mission'. Ses objectifs sociaux et environnementaux sont désormais inscrits dans ses statuts légaux.</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Argumentez en quoi cette décision constitue une évolution profonde de la finalité traditionnelle de l'entreprise face aux attentes de la société.</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>éthique | RSE | entreprise à mission | finalité | parties prenantes | gouvernance</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Argumentation : Traditionnellement, la finalité d'une entreprise privée est de maximiser le profit pour ses actionnaires. En devenant une 'Entreprise à mission' (loi PACTE), Danone modifie légalement sa raison d'être : la performance économique est désormais mise au même niveau que la performance sociale et environnementale. C'est une réponse structurelle forte : l'entreprise ne s'affranchit plus de son impact sur la société, elle accepte d'être auditée sur ses engagements (santé, climat) et d'en rendre compte à toutes ses parties prenantes, et non plus aux seuls financiers.</t>
+        </is>
+      </c>
+      <c r="M129" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>MT3-29</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>3.4. Quelles relations entre les organisations et leur écosystème ?</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>14</v>
+      </c>
+      <c r="G130" t="n">
+        <v>5</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Écosystème d'innovation Station F</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>À Paris, le campus Station F fondé par Xavier Niel héberge plus de 1000 start-ups. On y trouve également des bureaux de fonds d'investissement, de grandes entreprises comme LVMH, des experts comptables et des représentants de l'administration publique (French Tech).</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Élaborez un diagnostic sur la manière dont ce dispositif crée un écosystème d'affaires global et renforce le développement des jeunes entreprises.</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>écosystème d'affaires | innovation | start-up | synergies | réseau d'acteurs</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Diagnostic : Station F dépasse le simple incubateur pour former un écosystème d'affaires complet. L'agrégation physique d'acteurs extrêmement diversifiés (start-ups, grands groupes, financeurs, pouvoirs publics) lève les barrières à l'entrée. Les jeunes pousses bénéficient de synergies immédiates : financement rapide, mentorat par des leaders mondiaux (comme LVMH), accès simplifié aux aides publiques. Ce brassage d'idées et de capitaux sur un même territoire décuple l'agilité, la capacité d'innovation et le taux de survie de ces entreprises.</t>
+        </is>
+      </c>
+      <c r="M130" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>MT3-30</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>terminale</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Thème 3 : Les organisations et la société</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>3.1. Les organisations peuvent-elles s'affranchir des questions de société ?</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>15</v>
+      </c>
+      <c r="G131" t="n">
+        <v>5</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Diagnostic Éthique et RSE Amazon</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Amazon France met en avant sa création de milliers d'emplois locaux et sa promesse de devenir neutre en carbone. En parallèle, l'entreprise est accusée d'évasion fiscale agressive, de détruire le petit commerce de proximité et d'imposer des cadences infernales dans ses entrepôts.</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Construisez une argumentation nuancée pour évaluer la réalité de la démarche RSE d'Amazon face aux accusations de 'social washing' et 'greenwashing'.</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>éthique | RSE | social washing | optimisation fiscale | contradictions stratégiques</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Argumentation : D'un côté, Amazon a un impact positif indéniable sur l'écosystème territorial via la création d'emplois directs massifs et d'infrastructures. De l'autre côté, son modèle est traversé par de profondes contradictions éthiques. L'optimisation fiscale prive l'État de ressources (comportement non civique). Les conditions de travail dégradées contredisent ses discours sur la performance sociale. Enfin, son modèle ultra-logistique de surconsommation questionne son engagement écologique. On peut donc diagnostiquer une forme de social/green washing : les actions RSE d'Amazon, bien que réelles (panneaux solaires), peinent à compenser les externalités négatives structurelles de son business model global.</t>
+        </is>
+      </c>
+      <c r="M131" t="n">
+        <v>350</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>